<commit_message>
Astro power bank implementation
</commit_message>
<xml_diff>
--- a/astro-powerbank/altium/li-ion-1s-protection/Fabrication Files/BOM/Bill of Materials-li-ion-1s-protection.xlsx
+++ b/astro-powerbank/altium/li-ion-1s-protection/Fabrication Files/BOM/Bill of Materials-li-ion-1s-protection.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stason\Desktop\Projects\salt-energy\astro-powerbank\altium\li-ion-1s-protection\Fabrication Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A8AB35CF-5D3A-43A1-8130-EC06754F8A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{95F69CE5-012A-4C1B-B2C5-B55A6EF96BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12930" yWindow="210" windowWidth="21330" windowHeight="16560" xr2:uid="{5250F088-BD5F-4A19-984E-51819F6B6F0C}"/>
+    <workbookView xWindow="12930" yWindow="210" windowWidth="21330" windowHeight="16560" xr2:uid="{19E3CD69-7573-46F4-831C-93CD29F0CD90}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-li-ion-1s-pro" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -477,7 +477,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA549967-E726-489D-A385-CB8DD5C92918}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DAC75CE-A611-40AA-8CC2-4032CB7EE296}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -545,6 +545,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>